<commit_message>
Duplicate Analysis: update outputs 2026-01-30
</commit_message>
<xml_diff>
--- a/outputs/2026-01-30/email_reports/Sysco_France.xlsx
+++ b/outputs/2026-01-30/email_reports/Sysco_France.xlsx
@@ -467,10 +467,10 @@
         <v>597</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -61111,7 +61111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61239,65 +61239,73 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>14634</t>
+          <t>484769</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SAUCE SALADE BKE  BI 5 L X3</t>
+          <t>DIM SUM CREVETTES HACAO 1KG X6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Nominated</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>102150</t>
+          <t>220341</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SSA245BI5LX3BRAKE</t>
+          <t>484769</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>BRAKE</t>
+          <t>EUSHIRA</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>60000000000009</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>99999999999999</t>
+          <t>9999999999999</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>3308650146343</t>
+          <t>8888888888888</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -61307,17 +61315,17 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>99999999999999</t>
+          <t>9999999999999</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>GTIN Outer</t>
+          <t>GTIN Outer (both filled)</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>3308650146343</t>
+          <t>8888888888888</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -61339,58 +61347,54 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>60598</t>
+          <t>14634</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GB PUREE FRAISE 1KG X6</t>
+          <t>SAUCE SALADE BKE  BI 5 L X3</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Nominated</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>104257</t>
+          <t>102150</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>AFA1C6AA0</t>
+          <t>SSA245BI5LX3BRAKE</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>EUPCKER</t>
+          <t>BRAKE</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>L</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -61399,10 +61403,14 @@
           <t>99999999999999</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>3308650146343</t>
+        </is>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -61415,7 +61423,11 @@
           <t>GTIN Outer</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>3308650146343</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>PLACEHOLDER</t>
@@ -61435,12 +61447,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>60603</t>
+          <t>60598</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GB PUREE MANGUE 1KG X6</t>
+          <t>GB PUREE FRAISE 1KG X6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -61465,7 +61477,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>AMG0C6AA0</t>
+          <t>AFA1C6AA0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -61513,6 +61525,102 @@
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVE-CHARGE-MISCELLANEOUS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sysco_France</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>60603</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GB PUREE MANGUE 1KG X6</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Nominated</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>104257</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AMG0C6AA0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>EUPCKER</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>99999999999999</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>99999999999999</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>GTIN Outer</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
         <is>
           <t>PLACEHOLDER</t>
         </is>

</xml_diff>